<commit_message>
Switch hydrogel to the team's 500 um 1% calcium-alginate patch
- params.py: L_gel 500 um, porosity 0.99, mesh 14 nm (Grassi 2009); plain
  alginate binds neither active (R_V = R_F = 1; Freeman 2008)
- regenerate all 18 figures; fig08/fig10 re-laid out for the new ranges
- one patch now covers 7.2 h; longest change interval 21.8 h for every wound
  size (daily is 10% short); FGF2-G3 lasts 2-3 d without retention
- Interactive 1 JS solver and defaults updated to the alginate patch
- page text, captions, wet-lab list and conclusion updated; bundled register
  and code zip rebuilt
</commit_message>
<xml_diff>
--- a/code/constants_register.xlsx
+++ b/code/constants_register.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_physical" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_species" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_model1_gel" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_model2_tissue" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_model3_MD2" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_model4_signaling" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_model5_NO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_model6_closure" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_model7_design" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_legacy_sensing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="0_physical" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="1_species" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2_model1_gel" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="3_model2_tissue" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="4_model3_MD2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="5_model4_signaling" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="6_model5_NO" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="7_model6_closure" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="8_model7_design" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="9_legacy_sensing" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,13 +454,11 @@
           <t>Constant register - HKU iGEM 2026 dual-release wound patch (V3 model)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr">
         <is>
           <t>Generated from: igem_newest_long_version.pdf (V3, Oct 8 2026) + iGem Parameter Table (1).pdf</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr"/>
       <c r="E1" t="inlineStr">
         <is>
           <t>Tier legend:</t>
@@ -1843,7 +1841,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.015</v>
+        <v>0.05</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -1857,12 +1855,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>parameter table</t>
+          <t>team (2026-10-09)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>as-manufactured 5% GelMA</t>
+          <t>as-manufactured 1% w/v Ca-alginate (100 mM CaCl2, HBS pH 7.4), 500 um</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1876,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.618</v>
+        <v>0.99</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -1887,17 +1885,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>D</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10987139/</t>
+          <t>1% w/v polymer ~0.6% v/v</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>parameter table; 5% monomer concentration</t>
+          <t>replaces 5% GelMA value 0.618</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1911,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.27</v>
+        <v>1.005</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -1932,7 +1930,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>parameter table; consistent: 0.618^-0.5 = 1.272; fitted from release assay later</t>
+          <t>0.99^-0.5 = 1.005; fitted from release assay later</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1946,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -1957,24 +1955,24 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>doc sweep 5-50 nm</t>
+          <t>https://doi.org/10.3390/molecules14083003</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>needs measurement (Flory-Rehner or SAXS)</t>
+          <t>Grassi et al. 2009, 1% Ca-alginate: 14 nm mechanical, 26 nm from release; sweep 5-50 nm kept</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Gelatin chain radius</t>
+          <t>Polymer (alginate) chain radius</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1992,15 +1990,19 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>doc (Amsden 1998)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>Amsden obstruction scaling</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>alginate chain radius not measured; 0.6-2 nm changes H_F by &lt;= 6%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2014,7 +2016,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.957</v>
+        <v>0.976</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -2033,7 +2035,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>mild hindrance at xi = 10 nm</t>
+          <t>at xi = 14 nm</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2051,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.878</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -2066,7 +2068,11 @@
           <t>same</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>at xi = 14 nm</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2080,7 +2086,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.4e-06</v>
+        <v>4.37e-06</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -2099,7 +2105,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>doc baseline (10% gel, 500 um) used 3.25e-6</t>
+          <t>alginate 500 um; 95% release 10.8 min</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2121,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1.35e-06</v>
+        <v>1.85e-06</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -2134,7 +2140,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>doc baseline used 1.15e-6</t>
+          <t>alginate 500 um; 95% release 25.4 min</t>
         </is>
       </c>
     </row>
@@ -2230,12 +2236,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>LOCKED: no heparin</t>
+          <t>https://pubmed.ncbi.nlm.nih.gov/18462788/</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>both species linear Fickian; R_F = R_V = 1</t>
+          <t>LOCKED: plain alginate does not bind FGFs (Freeman et al. 2008, SPR); alginate-sulfate would (Kd 5-11 nM)</t>
         </is>
       </c>
     </row>
@@ -2265,12 +2271,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>LOCKED: no heparin / no sorption lever</t>
+          <t>LOCKED: alginate is hydrophilic</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>retention lever removed from design space</t>
+          <t>no V14 sorption; retention would need covalent tethering</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
16 Oct patch redesign; FGF2-G3 f_rel = 0.31 +/- 0.07 from the BCA fit
Patch redesign (2.5 mm 1% Ca-alginate, 3 mg/mL V14, 200 ng/mL FGF2-G3,
f_rel 0.5 / 0.15) with regenerated figures, interactives, register and
verify.py; adds check_params_sync.py and build_bundle.py.

FGF2-G3 released fraction then set to 0.31 +/- 0.07 (least-squares fit of
f_rel x Crank to the 30 Sep BCA 30-min read, was a 0.15 T4 estimate):
FGF2-G3 above EC50 for 5.4 d (was 4.5), tissue peak 32.8 ng/mL (was 15.9).
V14 numbers unchanged; V14 still sets the schedule.
</commit_message>
<xml_diff>
--- a/code/constants_register.xlsx
+++ b/code/constants_register.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>25</v>
+        <v>145</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -576,25 +576,29 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>D</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>flow-cytometry anchor / design knob</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+          <t>derived: 14 Oct 2026 flow panel (gate-frequency detection limit)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>REPLACES the earlier T4 guess of 25 uM. Chain: gate-frequency detection limit 27.8 % (two-sided t, n = 3) -&gt; 13.1 % occupancy drop at SIGMA_LOG = 0.7 (T4) -&gt; K_D,P &gt;= 10.08 uM (ONE-SIDED lower bound) -&gt; C_target = K_D,P (a-1) = 145 uM, the dose at which half the MD2 pool is LPS-bound (a = [L]/KD_L = 15.4). psi_50 = 1+a would be 165 uM. Because K_D,P is a lower bound, so is the target. See v3model.occupancy_from_gate.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Released fraction assumed</t>
+          <t>Released (mobile) fraction, V14</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>f_rel</t>
+          <t>f_rel_V</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -612,43 +616,150 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>doc</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+          <t>team estimate (2026-10-16)</t>
+        </is>
+      </c>
+      <c r="G3" s="2">
+        <f> f_mob: only f_rel x loading is free to diffuse; the remainder stays in the gel. Was 1 (whole dose mobile). Measure by release assay to completion.</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Released (mobile) fraction, FGF2-G3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>f_rel_F</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>BCA fit, 30 Sep assay (adopted 2026-10-16)</t>
+        </is>
+      </c>
+      <c r="G4" s="2">
+        <f> f_mob for FGF2-G3; remainder stays in the gel. 0.31 +/- 0.07 (SE): least-squares fit of f_rel x Crank to the 30-min BCA read (G03). Was 0.15 (team estimate). Assay near its noise floor: confirm by release assay to completion on a log time grid.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>V14 loading in the gel</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>C_V_load</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2213.1</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>uM</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>team design (2026-10-16)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>3 mg/mL total = 2213 uM; mobile (free) loading = f_rel_V x this = 1107 uM. Loaded at the solubility lower bound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>FGF2-G3 loading in the gel</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>C_F_load</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ng/mL</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>team design (2026-10-16)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>200 ng/mL total = 12.1 nM; mobile = f_rel_F x this = 62 ng/mL. Closure treated state requires tissue FGF2-G3 &gt;= EC50_F (0.5 ng/mL) over the top delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Dressing-change interval</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>reapply_interval_d</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>T4</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>standard clinical practice (daily dressing changes)</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>protocol knob for reapplication scenarios; single-patch effect window is only ~2.2 h above 25 uM (structural: 150 um reservoir drains through dermal sink)</t>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>protocol knob for reapplication scenarios; see Model 7 (dressing interval set by coverage per patch). UPDATED 2026-10-16 for the 2.5 mm / 3 mg/mL design.</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1714,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>V14 solubility ceiling</t>
+          <t>V14 solubility ceiling (lower bound)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1612,7 +1723,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>738</v>
+        <v>2213.1</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -1621,17 +1732,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>doc 9.5</t>
+          <t>team loading 3 mg/mL (2026-10-16)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>1 mg/mL assumed; MEASURE (saturation solubility in casting buffer)</t>
+          <t>3 mg/mL dissolved in the casting buffer = 2213 uM; LOWER BOUND on saturation solubility (was 1 mg/mL = 738 uM, T4 assumption). Saturation not yet measured.</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1952,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -1855,12 +1966,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>team (2026-10-09)</t>
+          <t>team (2026-10-16)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>as-manufactured 1% w/v Ca-alginate (100 mM CaCl2, HBS pH 7.4), 500 um</t>
+          <t>as-manufactured 1% w/v Ca-alginate (100 mM CaCl2, HBS pH 7.4), 2.5 mm (was 500 um until 2026-10-16)</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2216,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>alginate 500 um; 95% release 10.8 min</t>
+          <t>alginate 2.5 mm; 95% release 5.6 h</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2251,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>alginate 500 um; 95% release 25.4 min</t>
+          <t>alginate 2.5 mm; 95% release 14.8 h</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2517,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>parameter table</t>
+          <t>parameter table. NOTE: this is the eps_t that enters the loading inversion C_V0 &gt;= C_target eps_t delta/(f_rel eps_g L_gel). At eps_t = 0.8 and delta = 500 um the requirement is 117 uM free (f_rel = 1); setting eps_t = 1 (a conservative upper bound) gives 146 uM. The register value governs.</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3342,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>self-consistency CHECK, not an input; reproduced at band = 364 um</t>
+          <t>self-consistency CHECK, not an input; reproduced at mac_band = 364 um with q_chronic and k_scavenge as tabulated.</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3414,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>parameter table (updated range; doc used 3-10 s); autoxidation is 2nd order -&gt; report as range</t>
+          <t>parameter table (updated range; the doc previously used 3-10 s). TISSUE NO consumption, which sets the penetration depth L_d in the legacy sensing analysis. NOT the same quantity as k_scavenge below. Consumption is second order, so t_1/2 is concentration dependent -&gt; report as a range.</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3449,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>parameter table</t>
+          <t>parameter table. Autoxidation in CULTURE MEDIUM (t_1/2 = ln2/k = 69 s), which is what the in-vitro free-NO balance uses, since Model 5 is a well and not tissue. About two decades slower than t_half_NO above; do not interchange them. Only free NO scales with this -- cumulative nitrite does not.</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3681,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.005</v>
+        <v>0.0364</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -3589,7 +3700,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>band x q / k_scav sets baseline NO; 36 nM reproduced at 364 um</t>
+          <t>CALIBRATED: band x q / k_scav sets baseline NO; 0.0364 cm (364 um) is the depth that reproduces the 36 nM wound-NO figure. The earlier 0.005 cm gave 262 nM and so contradicted the very number it was calibrated against. Not used by any figure.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update wiki model content and figures
</commit_message>
<xml_diff>
--- a/code/constants_register.xlsx
+++ b/code/constants_register.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="2" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +19,7 @@
     <sheet name="9_legacy_sensing" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -36,8 +35,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -49,7 +50,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000279EE"/>
+        <fgColor rgb="FF0279EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,7 +76,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -439,7 +440,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -507,7 +508,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -555,7 +556,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="100.8" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Efficacious V14 concentration</t>
@@ -567,7 +568,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>145</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -581,12 +582,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>derived: 14 Oct 2026 flow panel (gate-frequency detection limit)</t>
+          <t>derived: 17 Oct 2026 positive-gate-frequency proxy</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>REPLACES the earlier T4 guess of 25 uM. Chain: gate-frequency detection limit 27.8 % (two-sided t, n = 3) -&gt; 13.1 % occupancy drop at SIGMA_LOG = 0.7 (T4) -&gt; K_D,P &gt;= 10.08 uM (ONE-SIDED lower bound) -&gt; C_target = K_D,P (a-1) = 145 uM, the dose at which half the MD2 pool is LPS-bound (a = [L]/KD_L = 15.4). psi_50 = 1+a would be 165 uM. Because K_D,P is a lower bound, so is the target. See v3model.occupancy_from_gate.</t>
+          <t>17 Oct 2026 flow panel: 21.34% positive-gate decrease at 25 uM (n=4/group, p=0.0186), used directly as a provisional K_D,P proxy (5.62 uM); C_target=K_D,P(a-1)=80.9 uM. Uncalibrated gate-frequency proxy; not a validated affinity.</t>
         </is>
       </c>
     </row>
@@ -619,10 +620,7 @@
           <t>team estimate (2026-10-16)</t>
         </is>
       </c>
-      <c r="G3" s="2">
-        <f> f_mob: only f_rel x loading is free to diffuse; the remainder stays in the gel. Was 1 (whole dose mobile). Measure by release assay to completion.</f>
-        <v/>
-      </c>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -636,7 +634,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.31</v>
+        <v>0.45</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -650,15 +648,16 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>BCA fit, 30 Sep assay (adopted 2026-10-16)</t>
-        </is>
-      </c>
-      <c r="G4" s="2">
-        <f> f_mob for FGF2-G3; remainder stays in the gel. 0.31 +/- 0.07 (SE): least-squares fit of f_rel x Crank to the 30-min BCA read (G03). Was 0.15 (team estimate). Assay near its noise floor: confirm by release assay to completion on a log time grid.</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
+          <t>Fit from BCA Updated.xlsx (30-min BCA read; samples at 60, 90, 120 min), 3 wells/timepoint. f_rel = 0.447, residual-based SE = 0.055; rounded to 0.45 +/- 0.06.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>PROVISIONAL model-scaled estimate. Assumes Positive FGF control represents full dose and tested gel thickness matches 2.5 mm model. Test thickness/buffer volume were not recorded; signal is near assay noise floor. Validate with a log-grid release assay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>V14 loading in the gel</t>
@@ -693,7 +692,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="43.2" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>FGF2-G3 loading in the gel</t>
@@ -728,7 +727,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="43.2" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Dressing-change interval</t>
@@ -775,7 +774,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -823,7 +822,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28.8" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Cellulose thickness</t>
@@ -858,7 +857,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="28.8" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Cellulose porosity</t>
@@ -928,7 +927,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>NorR background activity</t>
@@ -1068,7 +1067,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="28.8" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Max transcription rate</t>
@@ -1222,7 +1221,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -1334,7 +1333,7 @@
           <t>SI definition</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1383,7 +1382,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -1501,7 +1500,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="28.8" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Hydrodynamic radius V14</t>
@@ -1513,7 +1512,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.73</v>
+        <v>0.87</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -1532,11 +1531,11 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>globular-volume equivalent; doc correlation 0.87 nm is the sensitivity bound</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>fitted correlation a_h = 0.0515 M^0.392 (doc App. A); band 0.8-1.0 nm. 0.73 = anhydrous-sphere lower bound, not used</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Hydrodynamic radius FGF2-G3</t>
@@ -1548,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.68</v>
+        <v>2.34</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -1567,11 +1566,11 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>doc correlation 2.34 nm is the sensitivity bound</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>same correlation; band 1.9-2.4 nm (Wilkins ~2.0). 1.68 = anhydrous-sphere lower bound, not used</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="43.2" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Free diffusivity V14 (37 C)</t>
@@ -1583,7 +1582,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4.5e-06</v>
+        <v>3.6e-06</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -1592,21 +1591,21 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Stokes-Einstein from Rh_V14, eta</t>
+          <t>correlation consensus, doc App. A</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>doc correlation routes give 3.6e-6 (band 2.5-4.5e-6); discrepancy carried as sensitivity</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>consensus of 3 correlations (doc App. A); band 2.5-4.5e-6. Stokes-Einstein at the anhydrous radius 0.87 nm gives 4.5e-6: upper bound only</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28.8" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Free diffusivity FGF2-G3 (37 C)</t>
@@ -1618,7 +1617,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2e-06</v>
+        <v>1.5e-06</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -1627,21 +1626,21 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Stokes-Einstein from Rh_FGF2G3, eta</t>
+          <t>correlation consensus, doc App. A</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>doc correlation 1.5e-6 (band 1.3-1.7e-6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>same; band 1.3-1.7e-6. Stokes-Einstein at the anhydrous radius 1.68 nm gives 2.0e-6: upper bound only</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="43.2" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>V14 half-life (gel/tissue)</t>
@@ -1676,7 +1675,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="28.8" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>FGF2-G3 half-life (37 C)</t>
@@ -1711,7 +1710,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="43.2" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>V14 solubility ceiling (lower bound)</t>
@@ -1810,7 +1809,7 @@
           <t>doc App A / ExPASy</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1847,7 +1846,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="28.8" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>V14 MD2 affinity</t>
@@ -1858,7 +1857,9 @@
           <t>KD_P</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n"/>
+      <c r="C14" s="2" t="n">
+        <v>5.63e-09</v>
+      </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
           <t>mol/cm3</t>
@@ -1866,17 +1867,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>T4</t>
+          <t>D</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>pending flow cytometry</t>
+          <t>Derived proxy from specimen 3/7 flow panel, 16 Oct 2026; 25 uM V14, 1 uM FITC-LPS</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>NOT KNOWN - no sequence method; Models 3-5 run in scaled form (psi, a, gamma)</t>
+          <t>PROVISIONAL. Assumes gate-frequency ratio equals normalized theta_LPS ratio; this mapping is not established by Eq. (mfi). r=12.8271/16.3071=0.7866; KD_P=25/[(1+1/0.065)(1/r-1)]=5.63 uM. Single-dose proxy; confirm with FCS/MFI or LPS titration.</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1893,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -1940,7 +1941,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28.8" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Hydrogel thickness</t>
@@ -2045,7 +2046,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Mesh size</t>
@@ -2127,7 +2128,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.976</v>
+        <v>0.971</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -2146,7 +2147,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>at xi = 14 nm</t>
+          <t>at a_i = 0.87 nm (correlation), xi = 14 nm</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2163,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.889</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2182,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>at xi = 14 nm</t>
+          <t>at a_i = 2.34 nm (correlation), xi = 14 nm</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2198,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>4.37e-06</v>
+        <v>3.478e-06</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -2232,7 +2233,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1.85e-06</v>
+        <v>1.327e-06</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -2284,7 +2285,7 @@
           <t>ln2 / t_half_V14</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2321,7 +2322,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="28.8" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Heparin/HS site density</t>
@@ -2403,7 +2404,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -2486,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Tissue porosity</t>
@@ -2550,7 +2551,7 @@
           <t>Bruggeman eps^(-1/2)</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2686,7 +2687,7 @@
           <t>thermal/functional t1/2 proxy</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2723,7 +2724,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="28.8" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Microvascular clearance FGF2-G3</t>
@@ -2840,7 +2841,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -2888,7 +2889,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28.8" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>LPS-MD2 dissociation constant</t>
@@ -2923,7 +2924,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="28.8" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>MD2-TLR4 affinity</t>
@@ -2958,7 +2959,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="28.8" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Wound endotoxin load</t>
@@ -2993,7 +2994,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="28.8" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Total TLR4/MD2 density</t>
@@ -3040,7 +3041,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -3117,7 +3118,7 @@
           <t>parameter table (JBC)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3183,7 +3184,7 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3214,9 +3215,9 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="28.8" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Therapeutic p65 target</t>
@@ -3263,7 +3264,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -3311,7 +3312,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28.8" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Wound NO concentration (team)</t>
@@ -3381,7 +3382,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>NO half-life (normoxic tissue)</t>
@@ -3418,7 +3419,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>NO scavenging rate</t>
@@ -3560,7 +3561,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="28.8" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>iNOS catalytic rate (Griess)</t>
@@ -3634,7 +3635,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="28.8" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Max iNOS rate (acute)</t>
@@ -3669,7 +3670,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="57.6" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Macrophage band depth</t>
@@ -3735,7 +3736,7 @@
           <t>doc, tau 2-6 h</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3768,7 +3769,7 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3799,7 +3800,7 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3848,7 +3849,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -3896,7 +3897,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="28.8" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Fibroblast motility</t>
@@ -3931,7 +3932,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="28.8" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Carrying capacity</t>
@@ -3966,7 +3967,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="28.8" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Basal proliferation (chronic)</t>
@@ -4001,7 +4002,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="43.2" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Basal death (chronic)</t>
@@ -4071,7 +4072,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="28.8" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>FGF proliferative EC50</t>
@@ -4135,7 +4136,7 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4166,9 +4167,9 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
+      <c r="G9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="43.2" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Max death increment</t>
@@ -4232,7 +4233,7 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4263,9 +4264,9 @@
           <t>doc</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="28.8" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Effect-compartment rate</t>
@@ -4331,7 +4332,7 @@
           <t>doc grid 1-5 mm</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4362,7 +4363,7 @@
           <t>doc 50-100 um</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">

</xml_diff>